<commit_message>
updated branch with latest changes
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3171" uniqueCount="1357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3571" uniqueCount="1519">
   <si>
     <t>Run #</t>
   </si>
@@ -4082,6 +4082,492 @@
   </si>
   <si>
     <t>04/08/2026, 19:42:02</t>
+  </si>
+  <si>
+    <t>DA-MLI-068875216</t>
+  </si>
+  <si>
+    <t>04/08/2026, 19:59:17</t>
+  </si>
+  <si>
+    <t>DA-MLI-069001217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 14:22:17</t>
+  </si>
+  <si>
+    <t>CP-NI-069004217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 14:55:21</t>
+  </si>
+  <si>
+    <t>CP-NI-069005217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 14:57:05</t>
+  </si>
+  <si>
+    <t>CP-SC-069006217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 14:58:28</t>
+  </si>
+  <si>
+    <t>DA-MLI-069007217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:00:53</t>
+  </si>
+  <si>
+    <t>DA-MLI-069008217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:05:58</t>
+  </si>
+  <si>
+    <t>DA-MLI-069009217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:09:01</t>
+  </si>
+  <si>
+    <t>DA-MLI-069010217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:11:20</t>
+  </si>
+  <si>
+    <t>DA-MLI-069011217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:13:37</t>
+  </si>
+  <si>
+    <t>DA-MLI-069012217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:16:09</t>
+  </si>
+  <si>
+    <t>DA-MLI-069013217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:18:27</t>
+  </si>
+  <si>
+    <t>DA-MLI-069014217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:19:56</t>
+  </si>
+  <si>
+    <t>DA-MLI-069016217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:22:17</t>
+  </si>
+  <si>
+    <t>DA-MLI-069017217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:24:40</t>
+  </si>
+  <si>
+    <t>DA-MLI-069018217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:27:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-069019217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:29:33</t>
+  </si>
+  <si>
+    <t>DA-MLI-069020217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:32:14</t>
+  </si>
+  <si>
+    <t>DA-MLI-069021217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:34:36</t>
+  </si>
+  <si>
+    <t>DA-MLI-069022217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:36:58</t>
+  </si>
+  <si>
+    <t>DA-MLI-069023217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:39:18</t>
+  </si>
+  <si>
+    <t>DA-MLI-069024217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:41:55</t>
+  </si>
+  <si>
+    <t>DA-MLI-069025217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:44:12</t>
+  </si>
+  <si>
+    <t>DA-MLI-069026217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:45:53</t>
+  </si>
+  <si>
+    <t>DA-MLI-069027217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:48:14</t>
+  </si>
+  <si>
+    <t>DA-MLI-069028217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:50:40</t>
+  </si>
+  <si>
+    <t>DA-MLI-069029217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:53:11</t>
+  </si>
+  <si>
+    <t>DA-MLI-069030217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 15:58:12</t>
+  </si>
+  <si>
+    <t>CP-MLI-069031217</t>
+  </si>
+  <si>
+    <t>TC_REG_034_COMM | Create Claim on a live commercial policy and submit mandatory details</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:02:33</t>
+  </si>
+  <si>
+    <t>CP-MLI-069033217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:23:16</t>
+  </si>
+  <si>
+    <t>CP-MLI-069035217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:27:49</t>
+  </si>
+  <si>
+    <t>CP-MLI-069036217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:30:24</t>
+  </si>
+  <si>
+    <t>CP-MLI-069037217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:32:50</t>
+  </si>
+  <si>
+    <t>CP-MLI-069038217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:35:19</t>
+  </si>
+  <si>
+    <t>CP-MLI-069039217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:37:44</t>
+  </si>
+  <si>
+    <t>CP-MLI-069041217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:40:17</t>
+  </si>
+  <si>
+    <t>CP-MLI-069043217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:42:36</t>
+  </si>
+  <si>
+    <t>CP-MLI-069044217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:45:07</t>
+  </si>
+  <si>
+    <t>CP-MLI-069045217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:47:37</t>
+  </si>
+  <si>
+    <t>CP-MLI-069046217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:50:09</t>
+  </si>
+  <si>
+    <t>CP-MLI-069047217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:52:37</t>
+  </si>
+  <si>
+    <t>CP-MLI-069048217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:55:00</t>
+  </si>
+  <si>
+    <t>CP-MLI-069049217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:57:30</t>
+  </si>
+  <si>
+    <t>CP-MLI-069051217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 16:59:54</t>
+  </si>
+  <si>
+    <t>CP-MLI-069052217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 17:02:32</t>
+  </si>
+  <si>
+    <t>CP-MLI-069053217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 17:05:14</t>
+  </si>
+  <si>
+    <t>CP-MLI-069054217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 17:07:53</t>
+  </si>
+  <si>
+    <t>CP-MLI-069055217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 17:10:28</t>
+  </si>
+  <si>
+    <t>CP-MLI-069057217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 17:35:46</t>
+  </si>
+  <si>
+    <t>CP-MLI-069065217</t>
+  </si>
+  <si>
+    <t>05/08/2026, 18:08:53</t>
+  </si>
+  <si>
+    <t>DA-MLI-069247218</t>
+  </si>
+  <si>
+    <t>TC_REG_034 | Create Claim on a live policy, update Claim Information and complete claim</t>
+  </si>
+  <si>
+    <t>06/08/2026, 12:25:35</t>
+  </si>
+  <si>
+    <t>DA-MLI-069252218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 12:36:55</t>
+  </si>
+  <si>
+    <t>DA-MLI-069253218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 12:42:03</t>
+  </si>
+  <si>
+    <t>DA-MLI-069254218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 12:51:02</t>
+  </si>
+  <si>
+    <t>DA-MLI-069260218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 12:55:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-069261218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:01:55</t>
+  </si>
+  <si>
+    <t>DA-MLI-069262218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:09:09</t>
+  </si>
+  <si>
+    <t>DA-MLI-069263218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:15:00</t>
+  </si>
+  <si>
+    <t>DA-MLI-069264218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:19:10</t>
+  </si>
+  <si>
+    <t>DA-MLI-069265218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:28:45</t>
+  </si>
+  <si>
+    <t>DA-MLI-069266218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:36:15</t>
+  </si>
+  <si>
+    <t>DA-MLI-069267218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:39:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-069268218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:44:29</t>
+  </si>
+  <si>
+    <t>DA-MLI-069270218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:53:37</t>
+  </si>
+  <si>
+    <t>DA-MLI-069271218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 13:58:33</t>
+  </si>
+  <si>
+    <t>DA-MLI-069272218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 14:02:57</t>
+  </si>
+  <si>
+    <t>DA-MLI-069277218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 14:07:42</t>
+  </si>
+  <si>
+    <t>DA-MLI-069280218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 14:18:03</t>
+  </si>
+  <si>
+    <t>DA-MLI-069281218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 14:28:07</t>
+  </si>
+  <si>
+    <t>DA-MLI-069289218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 14:51:24</t>
+  </si>
+  <si>
+    <t>DA-MLI-069290218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 14:54:56</t>
+  </si>
+  <si>
+    <t>DA-MLI-069292218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 15:01:57</t>
+  </si>
+  <si>
+    <t>DA-MLI-069293218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 15:04:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-069294218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 15:10:44</t>
+  </si>
+  <si>
+    <t>DA-MLI-069295218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 15:14:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-069326218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 15:17:38</t>
+  </si>
+  <si>
+    <t>DA-MLI-069327218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 15:21:37</t>
+  </si>
+  <si>
+    <t>DA-MLI-069328218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 15:25:48</t>
+  </si>
+  <si>
+    <t>DA-MLI-069329218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 15:30:25</t>
+  </si>
+  <si>
+    <t>DA-MLI-069330218</t>
+  </si>
+  <si>
+    <t>06/08/2026, 15:41:06</t>
   </si>
 </sst>
 </file>
@@ -4515,7 +5001,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F634"/>
+  <dimension ref="A1:F714"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -17206,6 +17692,1606 @@
         <v>1356</v>
       </c>
     </row>
+    <row r="635" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A635" s="4">
+        <v>634</v>
+      </c>
+      <c r="B635" s="5" t="s">
+        <v>1357</v>
+      </c>
+      <c r="C635" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="D635" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E635" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F635" s="5" t="s">
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="636" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A636" s="2">
+        <v>635</v>
+      </c>
+      <c r="B636" s="3" t="s">
+        <v>1359</v>
+      </c>
+      <c r="C636" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D636" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E636" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F636" s="3" t="s">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="637" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A637" s="4">
+        <v>636</v>
+      </c>
+      <c r="B637" s="5" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C637" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D637" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E637" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F637" s="5" t="s">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="638" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A638" s="2">
+        <v>637</v>
+      </c>
+      <c r="B638" s="3" t="s">
+        <v>1363</v>
+      </c>
+      <c r="C638" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D638" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E638" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F638" s="3" t="s">
+        <v>1364</v>
+      </c>
+    </row>
+    <row r="639" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A639" s="4">
+        <v>638</v>
+      </c>
+      <c r="B639" s="5" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C639" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D639" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E639" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F639" s="5" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="640" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A640" s="2">
+        <v>639</v>
+      </c>
+      <c r="B640" s="3" t="s">
+        <v>1367</v>
+      </c>
+      <c r="C640" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D640" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E640" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F640" s="3" t="s">
+        <v>1368</v>
+      </c>
+    </row>
+    <row r="641" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A641" s="4">
+        <v>640</v>
+      </c>
+      <c r="B641" s="5" t="s">
+        <v>1369</v>
+      </c>
+      <c r="C641" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D641" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E641" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F641" s="5" t="s">
+        <v>1370</v>
+      </c>
+    </row>
+    <row r="642" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A642" s="2">
+        <v>641</v>
+      </c>
+      <c r="B642" s="3" t="s">
+        <v>1371</v>
+      </c>
+      <c r="C642" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D642" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E642" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F642" s="3" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="643" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A643" s="4">
+        <v>642</v>
+      </c>
+      <c r="B643" s="5" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C643" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D643" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E643" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F643" s="5" t="s">
+        <v>1374</v>
+      </c>
+    </row>
+    <row r="644" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A644" s="2">
+        <v>643</v>
+      </c>
+      <c r="B644" s="3" t="s">
+        <v>1375</v>
+      </c>
+      <c r="C644" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D644" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E644" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F644" s="3" t="s">
+        <v>1376</v>
+      </c>
+    </row>
+    <row r="645" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A645" s="4">
+        <v>644</v>
+      </c>
+      <c r="B645" s="5" t="s">
+        <v>1377</v>
+      </c>
+      <c r="C645" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D645" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E645" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F645" s="5" t="s">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="646" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A646" s="2">
+        <v>645</v>
+      </c>
+      <c r="B646" s="3" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C646" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D646" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E646" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F646" s="3" t="s">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="647" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A647" s="4">
+        <v>646</v>
+      </c>
+      <c r="B647" s="5" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C647" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D647" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E647" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F647" s="5" t="s">
+        <v>1382</v>
+      </c>
+    </row>
+    <row r="648" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A648" s="2">
+        <v>647</v>
+      </c>
+      <c r="B648" s="3" t="s">
+        <v>1383</v>
+      </c>
+      <c r="C648" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D648" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E648" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F648" s="3" t="s">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="649" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A649" s="4">
+        <v>648</v>
+      </c>
+      <c r="B649" s="5" t="s">
+        <v>1385</v>
+      </c>
+      <c r="C649" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D649" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E649" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F649" s="5" t="s">
+        <v>1386</v>
+      </c>
+    </row>
+    <row r="650" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A650" s="2">
+        <v>649</v>
+      </c>
+      <c r="B650" s="3" t="s">
+        <v>1387</v>
+      </c>
+      <c r="C650" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D650" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E650" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F650" s="3" t="s">
+        <v>1388</v>
+      </c>
+    </row>
+    <row r="651" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A651" s="4">
+        <v>650</v>
+      </c>
+      <c r="B651" s="5" t="s">
+        <v>1389</v>
+      </c>
+      <c r="C651" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D651" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E651" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F651" s="5" t="s">
+        <v>1390</v>
+      </c>
+    </row>
+    <row r="652" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A652" s="2">
+        <v>651</v>
+      </c>
+      <c r="B652" s="3" t="s">
+        <v>1391</v>
+      </c>
+      <c r="C652" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D652" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E652" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F652" s="3" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="653" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A653" s="4">
+        <v>652</v>
+      </c>
+      <c r="B653" s="5" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C653" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D653" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E653" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F653" s="5" t="s">
+        <v>1394</v>
+      </c>
+    </row>
+    <row r="654" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A654" s="2">
+        <v>653</v>
+      </c>
+      <c r="B654" s="3" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C654" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D654" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E654" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F654" s="3" t="s">
+        <v>1396</v>
+      </c>
+    </row>
+    <row r="655" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A655" s="4">
+        <v>654</v>
+      </c>
+      <c r="B655" s="5" t="s">
+        <v>1397</v>
+      </c>
+      <c r="C655" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D655" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E655" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F655" s="5" t="s">
+        <v>1398</v>
+      </c>
+    </row>
+    <row r="656" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A656" s="2">
+        <v>655</v>
+      </c>
+      <c r="B656" s="3" t="s">
+        <v>1399</v>
+      </c>
+      <c r="C656" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D656" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E656" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F656" s="3" t="s">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="657" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A657" s="4">
+        <v>656</v>
+      </c>
+      <c r="B657" s="5" t="s">
+        <v>1401</v>
+      </c>
+      <c r="C657" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D657" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E657" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F657" s="5" t="s">
+        <v>1402</v>
+      </c>
+    </row>
+    <row r="658" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A658" s="2">
+        <v>657</v>
+      </c>
+      <c r="B658" s="3" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C658" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D658" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E658" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F658" s="3" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="659" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A659" s="4">
+        <v>658</v>
+      </c>
+      <c r="B659" s="5" t="s">
+        <v>1405</v>
+      </c>
+      <c r="C659" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D659" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E659" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F659" s="5" t="s">
+        <v>1406</v>
+      </c>
+    </row>
+    <row r="660" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A660" s="2">
+        <v>659</v>
+      </c>
+      <c r="B660" s="3" t="s">
+        <v>1407</v>
+      </c>
+      <c r="C660" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D660" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E660" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F660" s="3" t="s">
+        <v>1408</v>
+      </c>
+    </row>
+    <row r="661" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A661" s="4">
+        <v>660</v>
+      </c>
+      <c r="B661" s="5" t="s">
+        <v>1409</v>
+      </c>
+      <c r="C661" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D661" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E661" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F661" s="5" t="s">
+        <v>1410</v>
+      </c>
+    </row>
+    <row r="662" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A662" s="2">
+        <v>661</v>
+      </c>
+      <c r="B662" s="3" t="s">
+        <v>1411</v>
+      </c>
+      <c r="C662" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D662" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E662" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F662" s="3" t="s">
+        <v>1412</v>
+      </c>
+    </row>
+    <row r="663" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A663" s="4">
+        <v>662</v>
+      </c>
+      <c r="B663" s="5" t="s">
+        <v>1413</v>
+      </c>
+      <c r="C663" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D663" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E663" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F663" s="5" t="s">
+        <v>1415</v>
+      </c>
+    </row>
+    <row r="664" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A664" s="2">
+        <v>663</v>
+      </c>
+      <c r="B664" s="3" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C664" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D664" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E664" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F664" s="3" t="s">
+        <v>1417</v>
+      </c>
+    </row>
+    <row r="665" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A665" s="4">
+        <v>664</v>
+      </c>
+      <c r="B665" s="5" t="s">
+        <v>1418</v>
+      </c>
+      <c r="C665" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D665" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E665" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F665" s="5" t="s">
+        <v>1419</v>
+      </c>
+    </row>
+    <row r="666" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A666" s="2">
+        <v>665</v>
+      </c>
+      <c r="B666" s="3" t="s">
+        <v>1420</v>
+      </c>
+      <c r="C666" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D666" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E666" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F666" s="3" t="s">
+        <v>1421</v>
+      </c>
+    </row>
+    <row r="667" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A667" s="4">
+        <v>666</v>
+      </c>
+      <c r="B667" s="5" t="s">
+        <v>1422</v>
+      </c>
+      <c r="C667" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D667" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E667" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F667" s="5" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="668" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A668" s="2">
+        <v>667</v>
+      </c>
+      <c r="B668" s="3" t="s">
+        <v>1424</v>
+      </c>
+      <c r="C668" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D668" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E668" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F668" s="3" t="s">
+        <v>1425</v>
+      </c>
+    </row>
+    <row r="669" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A669" s="4">
+        <v>668</v>
+      </c>
+      <c r="B669" s="5" t="s">
+        <v>1426</v>
+      </c>
+      <c r="C669" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D669" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E669" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F669" s="5" t="s">
+        <v>1427</v>
+      </c>
+    </row>
+    <row r="670" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A670" s="2">
+        <v>669</v>
+      </c>
+      <c r="B670" s="3" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C670" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D670" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E670" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F670" s="3" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="671" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A671" s="4">
+        <v>670</v>
+      </c>
+      <c r="B671" s="5" t="s">
+        <v>1430</v>
+      </c>
+      <c r="C671" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D671" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E671" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F671" s="5" t="s">
+        <v>1431</v>
+      </c>
+    </row>
+    <row r="672" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A672" s="2">
+        <v>671</v>
+      </c>
+      <c r="B672" s="3" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C672" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D672" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E672" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F672" s="3" t="s">
+        <v>1433</v>
+      </c>
+    </row>
+    <row r="673" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A673" s="4">
+        <v>672</v>
+      </c>
+      <c r="B673" s="5" t="s">
+        <v>1434</v>
+      </c>
+      <c r="C673" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D673" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E673" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F673" s="5" t="s">
+        <v>1435</v>
+      </c>
+    </row>
+    <row r="674" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A674" s="2">
+        <v>673</v>
+      </c>
+      <c r="B674" s="3" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C674" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D674" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E674" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F674" s="3" t="s">
+        <v>1437</v>
+      </c>
+    </row>
+    <row r="675" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A675" s="4">
+        <v>674</v>
+      </c>
+      <c r="B675" s="5" t="s">
+        <v>1438</v>
+      </c>
+      <c r="C675" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D675" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E675" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F675" s="5" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="676" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A676" s="2">
+        <v>675</v>
+      </c>
+      <c r="B676" s="3" t="s">
+        <v>1440</v>
+      </c>
+      <c r="C676" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D676" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E676" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F676" s="3" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="677" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A677" s="4">
+        <v>676</v>
+      </c>
+      <c r="B677" s="5" t="s">
+        <v>1442</v>
+      </c>
+      <c r="C677" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D677" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E677" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F677" s="5" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="678" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A678" s="2">
+        <v>677</v>
+      </c>
+      <c r="B678" s="3" t="s">
+        <v>1444</v>
+      </c>
+      <c r="C678" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D678" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E678" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F678" s="3" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="679" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A679" s="4">
+        <v>678</v>
+      </c>
+      <c r="B679" s="5" t="s">
+        <v>1446</v>
+      </c>
+      <c r="C679" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D679" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E679" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F679" s="5" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="680" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A680" s="2">
+        <v>679</v>
+      </c>
+      <c r="B680" s="3" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C680" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D680" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E680" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F680" s="3" t="s">
+        <v>1449</v>
+      </c>
+    </row>
+    <row r="681" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A681" s="4">
+        <v>680</v>
+      </c>
+      <c r="B681" s="5" t="s">
+        <v>1450</v>
+      </c>
+      <c r="C681" s="5" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D681" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E681" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F681" s="5" t="s">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="682" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A682" s="2">
+        <v>681</v>
+      </c>
+      <c r="B682" s="3" t="s">
+        <v>1452</v>
+      </c>
+      <c r="C682" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D682" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E682" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F682" s="3" t="s">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="683" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A683" s="4">
+        <v>682</v>
+      </c>
+      <c r="B683" s="5" t="s">
+        <v>1454</v>
+      </c>
+      <c r="C683" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D683" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E683" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F683" s="5" t="s">
+        <v>1455</v>
+      </c>
+    </row>
+    <row r="684" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A684" s="2">
+        <v>683</v>
+      </c>
+      <c r="B684" s="3" t="s">
+        <v>1456</v>
+      </c>
+      <c r="C684" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D684" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E684" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F684" s="3" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="685" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A685" s="4">
+        <v>684</v>
+      </c>
+      <c r="B685" s="5" t="s">
+        <v>1458</v>
+      </c>
+      <c r="C685" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D685" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E685" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F685" s="5" t="s">
+        <v>1460</v>
+      </c>
+    </row>
+    <row r="686" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A686" s="2">
+        <v>685</v>
+      </c>
+      <c r="B686" s="3" t="s">
+        <v>1461</v>
+      </c>
+      <c r="C686" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D686" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E686" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F686" s="3" t="s">
+        <v>1462</v>
+      </c>
+    </row>
+    <row r="687" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A687" s="4">
+        <v>686</v>
+      </c>
+      <c r="B687" s="5" t="s">
+        <v>1463</v>
+      </c>
+      <c r="C687" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D687" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E687" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F687" s="5" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="688" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A688" s="2">
+        <v>687</v>
+      </c>
+      <c r="B688" s="3" t="s">
+        <v>1465</v>
+      </c>
+      <c r="C688" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D688" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E688" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F688" s="3" t="s">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="689" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A689" s="4">
+        <v>688</v>
+      </c>
+      <c r="B689" s="5" t="s">
+        <v>1467</v>
+      </c>
+      <c r="C689" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D689" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E689" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F689" s="5" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="690" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A690" s="2">
+        <v>689</v>
+      </c>
+      <c r="B690" s="3" t="s">
+        <v>1469</v>
+      </c>
+      <c r="C690" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D690" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E690" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F690" s="3" t="s">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="691" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A691" s="4">
+        <v>690</v>
+      </c>
+      <c r="B691" s="5" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C691" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D691" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E691" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F691" s="5" t="s">
+        <v>1472</v>
+      </c>
+    </row>
+    <row r="692" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A692" s="2">
+        <v>691</v>
+      </c>
+      <c r="B692" s="3" t="s">
+        <v>1473</v>
+      </c>
+      <c r="C692" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D692" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E692" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F692" s="3" t="s">
+        <v>1474</v>
+      </c>
+    </row>
+    <row r="693" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A693" s="4">
+        <v>692</v>
+      </c>
+      <c r="B693" s="5" t="s">
+        <v>1475</v>
+      </c>
+      <c r="C693" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D693" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E693" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F693" s="5" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="694" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A694" s="2">
+        <v>693</v>
+      </c>
+      <c r="B694" s="3" t="s">
+        <v>1477</v>
+      </c>
+      <c r="C694" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D694" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E694" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F694" s="3" t="s">
+        <v>1478</v>
+      </c>
+    </row>
+    <row r="695" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A695" s="4">
+        <v>694</v>
+      </c>
+      <c r="B695" s="5" t="s">
+        <v>1479</v>
+      </c>
+      <c r="C695" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D695" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E695" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F695" s="5" t="s">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="696" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A696" s="2">
+        <v>695</v>
+      </c>
+      <c r="B696" s="3" t="s">
+        <v>1481</v>
+      </c>
+      <c r="C696" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D696" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E696" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F696" s="3" t="s">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="697" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A697" s="4">
+        <v>696</v>
+      </c>
+      <c r="B697" s="5" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C697" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D697" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E697" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F697" s="5" t="s">
+        <v>1484</v>
+      </c>
+    </row>
+    <row r="698" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A698" s="2">
+        <v>697</v>
+      </c>
+      <c r="B698" s="3" t="s">
+        <v>1485</v>
+      </c>
+      <c r="C698" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D698" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E698" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F698" s="3" t="s">
+        <v>1486</v>
+      </c>
+    </row>
+    <row r="699" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A699" s="4">
+        <v>698</v>
+      </c>
+      <c r="B699" s="5" t="s">
+        <v>1487</v>
+      </c>
+      <c r="C699" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D699" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E699" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F699" s="5" t="s">
+        <v>1488</v>
+      </c>
+    </row>
+    <row r="700" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A700" s="2">
+        <v>699</v>
+      </c>
+      <c r="B700" s="3" t="s">
+        <v>1489</v>
+      </c>
+      <c r="C700" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D700" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E700" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F700" s="3" t="s">
+        <v>1490</v>
+      </c>
+    </row>
+    <row r="701" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A701" s="4">
+        <v>700</v>
+      </c>
+      <c r="B701" s="5" t="s">
+        <v>1491</v>
+      </c>
+      <c r="C701" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D701" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E701" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F701" s="5" t="s">
+        <v>1492</v>
+      </c>
+    </row>
+    <row r="702" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A702" s="2">
+        <v>701</v>
+      </c>
+      <c r="B702" s="3" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C702" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D702" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E702" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F702" s="3" t="s">
+        <v>1494</v>
+      </c>
+    </row>
+    <row r="703" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A703" s="4">
+        <v>702</v>
+      </c>
+      <c r="B703" s="5" t="s">
+        <v>1495</v>
+      </c>
+      <c r="C703" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D703" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E703" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F703" s="5" t="s">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="704" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A704" s="2">
+        <v>703</v>
+      </c>
+      <c r="B704" s="3" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C704" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D704" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E704" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F704" s="3" t="s">
+        <v>1498</v>
+      </c>
+    </row>
+    <row r="705" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A705" s="4">
+        <v>704</v>
+      </c>
+      <c r="B705" s="5" t="s">
+        <v>1499</v>
+      </c>
+      <c r="C705" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D705" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E705" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F705" s="5" t="s">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="706" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A706" s="2">
+        <v>705</v>
+      </c>
+      <c r="B706" s="3" t="s">
+        <v>1501</v>
+      </c>
+      <c r="C706" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D706" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E706" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F706" s="3" t="s">
+        <v>1502</v>
+      </c>
+    </row>
+    <row r="707" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A707" s="4">
+        <v>706</v>
+      </c>
+      <c r="B707" s="5" t="s">
+        <v>1503</v>
+      </c>
+      <c r="C707" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D707" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E707" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F707" s="5" t="s">
+        <v>1504</v>
+      </c>
+    </row>
+    <row r="708" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A708" s="2">
+        <v>707</v>
+      </c>
+      <c r="B708" s="3" t="s">
+        <v>1505</v>
+      </c>
+      <c r="C708" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D708" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E708" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F708" s="3" t="s">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="709" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A709" s="4">
+        <v>708</v>
+      </c>
+      <c r="B709" s="5" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C709" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D709" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E709" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F709" s="5" t="s">
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="710" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A710" s="2">
+        <v>709</v>
+      </c>
+      <c r="B710" s="3" t="s">
+        <v>1509</v>
+      </c>
+      <c r="C710" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D710" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E710" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F710" s="3" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="711" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A711" s="4">
+        <v>710</v>
+      </c>
+      <c r="B711" s="5" t="s">
+        <v>1511</v>
+      </c>
+      <c r="C711" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D711" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E711" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F711" s="5" t="s">
+        <v>1512</v>
+      </c>
+    </row>
+    <row r="712" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A712" s="2">
+        <v>711</v>
+      </c>
+      <c r="B712" s="3" t="s">
+        <v>1513</v>
+      </c>
+      <c r="C712" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D712" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E712" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F712" s="3" t="s">
+        <v>1514</v>
+      </c>
+    </row>
+    <row r="713" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A713" s="4">
+        <v>712</v>
+      </c>
+      <c r="B713" s="5" t="s">
+        <v>1515</v>
+      </c>
+      <c r="C713" s="5" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D713" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E713" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F713" s="5" t="s">
+        <v>1516</v>
+      </c>
+    </row>
+    <row r="714" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A714" s="2">
+        <v>713</v>
+      </c>
+      <c r="B714" s="3" t="s">
+        <v>1517</v>
+      </c>
+      <c r="C714" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D714" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E714" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F714" s="3" t="s">
+        <v>1518</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
Add remaining local updates and generated reports
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4906" uniqueCount="2085">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4956" uniqueCount="2107">
   <si>
     <t>Run #</t>
   </si>
@@ -6269,6 +6269,72 @@
   </si>
   <si>
     <t>25/09/2026, 18:34:00</t>
+  </si>
+  <si>
+    <t>CP-MLI-631334268</t>
+  </si>
+  <si>
+    <t>25/09/2026, 19:44:08</t>
+  </si>
+  <si>
+    <t>CP-MLI-631335268</t>
+  </si>
+  <si>
+    <t>25/09/2026, 19:52:23</t>
+  </si>
+  <si>
+    <t>CP-MLI-631336268</t>
+  </si>
+  <si>
+    <t>25/09/2026, 20:01:58</t>
+  </si>
+  <si>
+    <t>CP-MLI-631337268</t>
+  </si>
+  <si>
+    <t>25/09/2026, 20:26:51</t>
+  </si>
+  <si>
+    <t>CP-MLI-556211271</t>
+  </si>
+  <si>
+    <t>Create commercial England and Wales policy with four products</t>
+  </si>
+  <si>
+    <t>28/09/2026, 14:02:24</t>
+  </si>
+  <si>
+    <t>CP-MLI-556215271</t>
+  </si>
+  <si>
+    <t>28/09/2026, 15:12:17</t>
+  </si>
+  <si>
+    <t>DA-MLI-556223271</t>
+  </si>
+  <si>
+    <t>Cancel policy from inception after creating a fresh live policy</t>
+  </si>
+  <si>
+    <t>28/09/2026, 15:49:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-556225271</t>
+  </si>
+  <si>
+    <t>28/09/2026, 16:10:42</t>
+  </si>
+  <si>
+    <t>DA-MLI-631413271</t>
+  </si>
+  <si>
+    <t>28/09/2026, 16:43:27</t>
+  </si>
+  <si>
+    <t>DA-MLI-631414271</t>
+  </si>
+  <si>
+    <t>28/09/2026, 16:48:45</t>
   </si>
 </sst>
 </file>
@@ -6742,7 +6808,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F981"/>
+  <dimension ref="A1:F991"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -26373,6 +26439,206 @@
         <v>2084</v>
       </c>
     </row>
+    <row r="982" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A982" s="11">
+        <v>981</v>
+      </c>
+      <c r="B982" s="12" t="s">
+        <v>2085</v>
+      </c>
+      <c r="C982" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D982" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E982" s="12" t="s">
+        <v>2009</v>
+      </c>
+      <c r="F982" s="12" t="s">
+        <v>2086</v>
+      </c>
+    </row>
+    <row r="983" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A983" s="13">
+        <v>982</v>
+      </c>
+      <c r="B983" s="14" t="s">
+        <v>2087</v>
+      </c>
+      <c r="C983" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D983" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E983" s="14" t="s">
+        <v>2009</v>
+      </c>
+      <c r="F983" s="14" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="984" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A984" s="11">
+        <v>983</v>
+      </c>
+      <c r="B984" s="12" t="s">
+        <v>2089</v>
+      </c>
+      <c r="C984" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D984" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E984" s="12" t="s">
+        <v>2009</v>
+      </c>
+      <c r="F984" s="12" t="s">
+        <v>2090</v>
+      </c>
+    </row>
+    <row r="985" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A985" s="13">
+        <v>984</v>
+      </c>
+      <c r="B985" s="14" t="s">
+        <v>2091</v>
+      </c>
+      <c r="C985" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D985" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E985" s="14" t="s">
+        <v>2009</v>
+      </c>
+      <c r="F985" s="14" t="s">
+        <v>2092</v>
+      </c>
+    </row>
+    <row r="986" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A986" s="11">
+        <v>985</v>
+      </c>
+      <c r="B986" s="12" t="s">
+        <v>2093</v>
+      </c>
+      <c r="C986" s="12" t="s">
+        <v>2094</v>
+      </c>
+      <c r="D986" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E986" s="12" t="s">
+        <v>491</v>
+      </c>
+      <c r="F986" s="12" t="s">
+        <v>2095</v>
+      </c>
+    </row>
+    <row r="987" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A987" s="13">
+        <v>986</v>
+      </c>
+      <c r="B987" s="14" t="s">
+        <v>2096</v>
+      </c>
+      <c r="C987" s="14" t="s">
+        <v>2094</v>
+      </c>
+      <c r="D987" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E987" s="14" t="s">
+        <v>491</v>
+      </c>
+      <c r="F987" s="14" t="s">
+        <v>2097</v>
+      </c>
+    </row>
+    <row r="988" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A988" s="11">
+        <v>987</v>
+      </c>
+      <c r="B988" s="12" t="s">
+        <v>2098</v>
+      </c>
+      <c r="C988" s="12" t="s">
+        <v>2099</v>
+      </c>
+      <c r="D988" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E988" s="12" t="s">
+        <v>491</v>
+      </c>
+      <c r="F988" s="12" t="s">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="989" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A989" s="13">
+        <v>988</v>
+      </c>
+      <c r="B989" s="14" t="s">
+        <v>2101</v>
+      </c>
+      <c r="C989" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="D989" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E989" s="14" t="s">
+        <v>491</v>
+      </c>
+      <c r="F989" s="14" t="s">
+        <v>2102</v>
+      </c>
+    </row>
+    <row r="990" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A990" s="11">
+        <v>989</v>
+      </c>
+      <c r="B990" s="12" t="s">
+        <v>2103</v>
+      </c>
+      <c r="C990" s="12" t="s">
+        <v>2053</v>
+      </c>
+      <c r="D990" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E990" s="12" t="s">
+        <v>2009</v>
+      </c>
+      <c r="F990" s="12" t="s">
+        <v>2104</v>
+      </c>
+    </row>
+    <row r="991" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A991" s="13">
+        <v>990</v>
+      </c>
+      <c r="B991" s="14" t="s">
+        <v>2105</v>
+      </c>
+      <c r="C991" s="14" t="s">
+        <v>2053</v>
+      </c>
+      <c r="D991" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E991" s="14" t="s">
+        <v>2009</v>
+      </c>
+      <c r="F991" s="14" t="s">
+        <v>2106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add TC_REG_061 residential E2E flow and orchestrator/reporting updates
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4956" uniqueCount="2107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4961" uniqueCount="2110">
   <si>
     <t>Run #</t>
   </si>
@@ -6335,6 +6335,15 @@
   </si>
   <si>
     <t>28/09/2026, 16:48:45</t>
+  </si>
+  <si>
+    <t>DA-MLI-556256272</t>
+  </si>
+  <si>
+    <t>TC_REG_061 | Create Residential England &amp; Wales policy (end-to-end)</t>
+  </si>
+  <si>
+    <t>29/09/2026, 16:18:53</t>
   </si>
 </sst>
 </file>
@@ -6808,7 +6817,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F991"/>
+  <dimension ref="A1:F992"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -26639,6 +26648,26 @@
         <v>2106</v>
       </c>
     </row>
+    <row r="992" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A992" s="11">
+        <v>991</v>
+      </c>
+      <c r="B992" s="12" t="s">
+        <v>2107</v>
+      </c>
+      <c r="C992" s="12" t="s">
+        <v>2108</v>
+      </c>
+      <c r="D992" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E992" s="12" t="s">
+        <v>491</v>
+      </c>
+      <c r="F992" s="12" t="s">
+        <v>2109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>